<commit_message>
Backup A: 2026-05-26 22:00
</commit_message>
<xml_diff>
--- a/media/课外班课程表.xlsx
+++ b/media/课外班课程表.xlsx
@@ -30,16 +30,16 @@
       <name val="微软雅黑"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="16"/>
     </font>
     <font>
       <name val="微软雅黑"/>
       <b val="1"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="微软雅黑"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -459,14 +459,14 @@
   <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>蛋蛋（盛泽扬）- 初二 13岁 课外班课程表</t>
@@ -706,14 +706,14 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>妞妞（李沐甜）- 小学一年级 6岁 课外班课程表</t>

</xml_diff>